<commit_message>
Register odoslane: doplnene datumy dokumentov (stlpec Datum)
</commit_message>
<xml_diff>
--- a/sud-landshut-telekom/odoslane/FIA_LG_Landshut_dokumenty_zoznam_suborov_odoslane.xlsx
+++ b/sud-landshut-telekom/odoslane/FIA_LG_Landshut_dokumenty_zoznam_suborov_odoslane.xlsx
@@ -600,7 +600,11 @@
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>02.10.2024</t>
+        </is>
+      </c>
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
@@ -627,7 +631,11 @@
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>17.10.2024</t>
+        </is>
+      </c>
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
@@ -654,7 +662,11 @@
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>14.11.2024</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
@@ -723,7 +735,11 @@
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>14.11.2024</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
@@ -750,7 +766,11 @@
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>04.12.2024</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
@@ -777,7 +797,11 @@
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>07.12.2024</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
@@ -804,7 +828,11 @@
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>07.12.2024</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
@@ -831,7 +859,11 @@
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>10.12.2024</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
@@ -858,7 +890,11 @@
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>10.12.2024</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
@@ -885,7 +921,11 @@
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>11.12.2024</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
@@ -912,7 +952,11 @@
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>11.12.2024</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="5" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
@@ -935,7 +979,11 @@
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>11.12.2024</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
@@ -962,7 +1010,11 @@
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
-      <c r="G16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>12.12.2024</t>
+        </is>
+      </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
@@ -989,7 +1041,11 @@
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>12.12.2024</t>
+        </is>
+      </c>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
@@ -1012,7 +1068,11 @@
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>12.12.2024</t>
+        </is>
+      </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="5" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
@@ -1039,7 +1099,11 @@
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>12.12.2024</t>
+        </is>
+      </c>
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="5" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
@@ -1066,7 +1130,11 @@
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>13.12.2024</t>
+        </is>
+      </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="5" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
@@ -1093,7 +1161,11 @@
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>13.12.2024</t>
+        </is>
+      </c>
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
@@ -1120,7 +1192,11 @@
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>14.12.2024</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
@@ -1147,7 +1223,11 @@
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr"/>
-      <c r="G23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>15.12.2024</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="5" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
@@ -1174,7 +1254,11 @@
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr"/>
-      <c r="G24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>17.12.2024</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
@@ -1201,7 +1285,11 @@
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr"/>
-      <c r="G25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>20.12.2024</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="5" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
@@ -1224,7 +1312,11 @@
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
-      <c r="G26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>22.12.2024</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="5" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
@@ -1251,7 +1343,11 @@
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
-      <c r="G27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>23.12.2024</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="5" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
@@ -1278,7 +1374,11 @@
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>14.01.2025</t>
+        </is>
+      </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="5" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
@@ -1305,7 +1405,11 @@
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr"/>
-      <c r="G29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>15.01.2025</t>
+        </is>
+      </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="5" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
@@ -1332,7 +1436,11 @@
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>17.01.2025</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="5" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
@@ -1359,7 +1467,11 @@
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>17.01.2025</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="5" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
@@ -1403,7 +1515,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1524,7 +1635,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>

</xml_diff>